<commit_message>
On branch main  Changes to be committed: 	modified:   wishlist.xlsx
</commit_message>
<xml_diff>
--- a/wishlist.xlsx
+++ b/wishlist.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/badf9f117d962842/Stalzone/Stalzone economic analyze/deal_bot/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="11_8A4311DF944722FE66105C1447739EFA0E228B27" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BAF379CB-75F8-42AA-A257-7AB4A6FAAD39}"/>
+  <xr:revisionPtr revIDLastSave="33" documentId="11_8A4311DF944722FE66105C1447739EFA0E228B27" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B4E5C96F-6A47-40DD-8F58-4A87E6C87F0E}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
   <si>
     <t>id</t>
   </si>
@@ -104,13 +104,34 @@
   </si>
   <si>
     <t>g4lzg</t>
+  </si>
+  <si>
+    <t>gmy0</t>
+  </si>
+  <si>
+    <t>Очищающий реагент</t>
+  </si>
+  <si>
+    <t>qokj</t>
+  </si>
+  <si>
+    <t>Тыква</t>
+  </si>
+  <si>
+    <t>knm0v</t>
+  </si>
+  <si>
+    <t>СВ-98</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+  </numFmts>
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -133,6 +154,13 @@
       <sz val="9"/>
       <color rgb="FF666666"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -177,10 +205,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -192,8 +221,18 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="2" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -498,7 +537,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -631,18 +670,54 @@
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
     </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" s="7">
+        <v>600000</v>
+      </c>
+      <c r="D13" s="5">
+        <v>0.1</v>
+      </c>
+    </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="C15" s="7">
+        <v>1800000</v>
+      </c>
+      <c r="D15" s="5"/>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A17" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" s="4" t="s">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A18" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A16" s="4" t="s">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A19" s="4" t="s">
         <v>16</v>
       </c>
     </row>

</xml_diff>